<commit_message>
fix(catalogo): ferramentas — produto compra vs comp2 (fita, talhadeira, prumo…)
- Core: 18 SKUs em Ferramentas com produto_compra e novo_sku corrigidos
- FITA genérico desdobrado via sku legado (VEDA ROSCA, ZEBRADA, SILVER TAPE…)
- Talhadeira, régua, marreta, linha de pedreiro e prumos Ramada normalizados
- Regenerados Excel 4×3 e PDFs

Co-authored-by: joaoandreriberopacheco-netizen <joaoandreriberopacheco-netizen@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/exports/P38-sku-hierarquia-core.xlsx
+++ b/docs/exports/P38-sku-hierarquia-core.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10946" uniqueCount="4119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10946" uniqueCount="4118">
   <si>
     <t>codigo_interno</t>
   </si>
@@ -11140,15 +11140,12 @@
     <t>1NB-OOL</t>
   </si>
   <si>
-    <t>FITA</t>
+    <t>FITA ALTA TENSÃO</t>
   </si>
   <si>
     <t>5M</t>
   </si>
   <si>
-    <t>FITA 5M</t>
-  </si>
-  <si>
     <t>FITA ALTA TENSÃO 5M</t>
   </si>
   <si>
@@ -11248,12 +11245,12 @@
     <t>UIR-OJ2</t>
   </si>
   <si>
+    <t>FITA DUPLA FACE</t>
+  </si>
+  <si>
     <t>12MMX2M</t>
   </si>
   <si>
-    <t>FITA 12MMX2M ADELBRAS</t>
-  </si>
-  <si>
     <t>FITA DUPLA FACE 12MMX2M ADELBRAS</t>
   </si>
   <si>
@@ -11290,19 +11287,19 @@
     <t>GTW-XH0</t>
   </si>
   <si>
+    <t>FITA SILVER TAPE</t>
+  </si>
+  <si>
     <t>48MM X 25M</t>
   </si>
   <si>
-    <t>FITA 48MM X 25M TEKBOND</t>
-  </si>
-  <si>
     <t>FITA SILVER TAPE 48MM X 25M TEKBOND</t>
   </si>
   <si>
     <t>IU5-V5A</t>
   </si>
   <si>
-    <t>FITA 18MM X 50M</t>
+    <t>FITA VEDA ROSCA</t>
   </si>
   <si>
     <t>FITA VEDA ROSCA 18MM X 50M</t>
@@ -11314,9 +11311,6 @@
     <t>18MM X 10M</t>
   </si>
   <si>
-    <t>FITA 18MM X 10M</t>
-  </si>
-  <si>
     <t>FITA VEDA ROSCA 18MM X 10M</t>
   </si>
   <si>
@@ -11326,21 +11320,18 @@
     <t>18MM X 25M</t>
   </si>
   <si>
-    <t>FITA 18MM X 25M</t>
-  </si>
-  <si>
     <t>FITA VEDA ROSCA 18MM X 25M</t>
   </si>
   <si>
     <t>BCG-YS0</t>
   </si>
   <si>
+    <t>FITA ZEBRADA</t>
+  </si>
+  <si>
     <t>100M</t>
   </si>
   <si>
-    <t>FITA 100M</t>
-  </si>
-  <si>
     <t>FITA ZEBRADA 100M</t>
   </si>
   <si>
@@ -11350,9 +11341,6 @@
     <t>50M</t>
   </si>
   <si>
-    <t>FITA 50M</t>
-  </si>
-  <si>
     <t>FITA ZEBRADA 50M</t>
   </si>
   <si>
@@ -11428,12 +11416,12 @@
     <t>IS6-TWG</t>
   </si>
   <si>
-    <t>LINHA DE PEDREIRO 50M</t>
-  </si>
-  <si>
     <t>50 M</t>
   </si>
   <si>
+    <t>LINHA DE PEDREIRO 50 M</t>
+  </si>
+  <si>
     <t>LINHA DE PEDREIRO 50M 50 M</t>
   </si>
   <si>
@@ -11755,25 +11743,25 @@
     <t>016-94X</t>
   </si>
   <si>
+    <t>MARRETA OITAVADA C/CABO</t>
+  </si>
+  <si>
+    <t>1,50KG</t>
+  </si>
+  <si>
+    <t>MARRETA OITAVADA C/CABO 1,50KG</t>
+  </si>
+  <si>
     <t>MARRETA OITAVADA 1,50KG C/CABO</t>
   </si>
   <si>
-    <t>1,50KG</t>
-  </si>
-  <si>
-    <t>MARRETA OITAVADA 1,50KG C/CABO 1,50KG</t>
-  </si>
-  <si>
     <t>F99-KB2</t>
   </si>
   <si>
-    <t>MARRETA OITAVADA 3KG C/CABO</t>
-  </si>
-  <si>
     <t>3KG</t>
   </si>
   <si>
-    <t>MARRETA OITAVADA 3KG C/CABO 3KG</t>
+    <t>MARRETA OITAVADA C/CABO 3KG</t>
   </si>
   <si>
     <t>MARRETA OITAVADA 3KG C/CABO MOMFORT</t>
@@ -12082,19 +12070,22 @@
     <t>BJU-Y8R</t>
   </si>
   <si>
-    <t>PRUMO HOBBY DE CENTRO</t>
+    <t>PRUMO DE CENTRO HOBBY RAMADA</t>
   </si>
   <si>
     <t>300G</t>
   </si>
   <si>
+    <t>PRUMO DE CENTRO HOBBY RAMADA 300G</t>
+  </si>
+  <si>
     <t>PRUMO HOBBY DE CENTRO 300G</t>
   </si>
   <si>
     <t>34N-6NP</t>
   </si>
   <si>
-    <t>PRUMO PAREDE HOBBY RAMADA</t>
+    <t>PRUMO DE PAREDE HOBBY RAMADA</t>
   </si>
   <si>
     <t>PRUMO PAREDE HOBBY RAMADA 3854</t>
@@ -12103,27 +12094,30 @@
     <t>DN0-8DH</t>
   </si>
   <si>
+    <t>RÉGUA DE PEDREIRO</t>
+  </si>
+  <si>
+    <t>2 M</t>
+  </si>
+  <si>
+    <t>RÉGUA DE PEDREIRO 2 M</t>
+  </si>
+  <si>
     <t>RÉGUA PEDREIRO 2 M</t>
   </si>
   <si>
-    <t>2 M</t>
-  </si>
-  <si>
-    <t>RÉGUA PEDREIRO 2 M 2 M</t>
-  </si>
-  <si>
     <t>0R4-XH1</t>
   </si>
   <si>
+    <t>3 M</t>
+  </si>
+  <si>
+    <t>RÉGUA DE PEDREIRO 3 M</t>
+  </si>
+  <si>
     <t>RÉGUA PEDREIRO 3 M</t>
   </si>
   <si>
-    <t>3 M</t>
-  </si>
-  <si>
-    <t>RÉGUA PEDREIRO 3 M 3 M</t>
-  </si>
-  <si>
     <t>K9O-WKV</t>
   </si>
   <si>
@@ -12179,6 +12173,9 @@
   </si>
   <si>
     <t>Z0Z-E1J</t>
+  </si>
+  <si>
+    <t>TALHADEIRA CHATA</t>
   </si>
   <si>
     <t>TALHADEIRA CHATA 8</t>
@@ -43849,12 +43846,12 @@
         <v>3710</v>
       </c>
       <c r="I1072" t="s">
-        <v>3711</v>
+        <v>3710</v>
       </c>
     </row>
     <row r="1073" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1073" t="s">
-        <v>3712</v>
+        <v>3711</v>
       </c>
       <c r="B1073" t="s">
         <v>66</v>
@@ -43866,24 +43863,24 @@
         <v>3423</v>
       </c>
       <c r="E1073" t="s">
+        <v>3712</v>
+      </c>
+      <c r="F1073" t="s">
         <v>3713</v>
       </c>
-      <c r="F1073" t="s">
+      <c r="G1073" t="s">
         <v>3714</v>
       </c>
-      <c r="G1073" t="s">
+      <c r="H1073" t="s">
         <v>3715</v>
       </c>
-      <c r="H1073" t="s">
+      <c r="I1073" t="s">
         <v>3716</v>
-      </c>
-      <c r="I1073" t="s">
-        <v>3717</v>
       </c>
     </row>
     <row r="1074" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1074" t="s">
-        <v>3718</v>
+        <v>3717</v>
       </c>
       <c r="B1074" t="s">
         <v>66</v>
@@ -43895,24 +43892,24 @@
         <v>3423</v>
       </c>
       <c r="E1074" t="s">
-        <v>3713</v>
+        <v>3712</v>
       </c>
       <c r="F1074" t="s">
         <v>3668</v>
       </c>
       <c r="G1074" t="s">
-        <v>3715</v>
+        <v>3714</v>
       </c>
       <c r="H1074" t="s">
+        <v>3718</v>
+      </c>
+      <c r="I1074" t="s">
         <v>3719</v>
-      </c>
-      <c r="I1074" t="s">
-        <v>3720</v>
       </c>
     </row>
     <row r="1075" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1075" t="s">
-        <v>3721</v>
+        <v>3720</v>
       </c>
       <c r="B1075" t="s">
         <v>66</v>
@@ -43924,24 +43921,24 @@
         <v>3423</v>
       </c>
       <c r="E1075" t="s">
-        <v>3713</v>
+        <v>3712</v>
       </c>
       <c r="F1075" t="s">
+        <v>3721</v>
+      </c>
+      <c r="G1075" t="s">
+        <v>3714</v>
+      </c>
+      <c r="H1075" t="s">
         <v>3722</v>
       </c>
-      <c r="G1075" t="s">
-        <v>3715</v>
-      </c>
-      <c r="H1075" t="s">
+      <c r="I1075" t="s">
         <v>3723</v>
-      </c>
-      <c r="I1075" t="s">
-        <v>3724</v>
       </c>
     </row>
     <row r="1076" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1076" t="s">
-        <v>3725</v>
+        <v>3724</v>
       </c>
       <c r="B1076" t="s">
         <v>66</v>
@@ -43953,24 +43950,24 @@
         <v>3423</v>
       </c>
       <c r="E1076" t="s">
+        <v>3725</v>
+      </c>
+      <c r="F1076" t="s">
         <v>3726</v>
-      </c>
-      <c r="F1076" t="s">
-        <v>3727</v>
       </c>
       <c r="G1076" t="s">
         <v>2305</v>
       </c>
       <c r="H1076" t="s">
-        <v>3728</v>
+        <v>3727</v>
       </c>
       <c r="I1076" t="s">
-        <v>3728</v>
+        <v>3727</v>
       </c>
     </row>
     <row r="1077" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1077" t="s">
-        <v>3729</v>
+        <v>3728</v>
       </c>
       <c r="B1077" t="s">
         <v>66</v>
@@ -43982,24 +43979,24 @@
         <v>3423</v>
       </c>
       <c r="E1077" t="s">
+        <v>3725</v>
+      </c>
+      <c r="F1077" t="s">
         <v>3726</v>
       </c>
-      <c r="F1077" t="s">
-        <v>3727</v>
-      </c>
       <c r="G1077" t="s">
+        <v>3729</v>
+      </c>
+      <c r="H1077" t="s">
         <v>3730</v>
       </c>
-      <c r="H1077" t="s">
-        <v>3731</v>
-      </c>
       <c r="I1077" t="s">
-        <v>3731</v>
+        <v>3730</v>
       </c>
     </row>
     <row r="1078" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1078" t="s">
-        <v>3732</v>
+        <v>3731</v>
       </c>
       <c r="B1078" t="s">
         <v>66</v>
@@ -44011,24 +44008,24 @@
         <v>3423</v>
       </c>
       <c r="E1078" t="s">
+        <v>3725</v>
+      </c>
+      <c r="F1078" t="s">
         <v>3726</v>
-      </c>
-      <c r="F1078" t="s">
-        <v>3727</v>
       </c>
       <c r="G1078" t="s">
         <v>3703</v>
       </c>
       <c r="H1078" t="s">
-        <v>3733</v>
+        <v>3732</v>
       </c>
       <c r="I1078" t="s">
-        <v>3733</v>
+        <v>3732</v>
       </c>
     </row>
     <row r="1079" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1079" t="s">
-        <v>3734</v>
+        <v>3733</v>
       </c>
       <c r="B1079" t="s">
         <v>66</v>
@@ -44040,24 +44037,24 @@
         <v>3423</v>
       </c>
       <c r="E1079" t="s">
-        <v>3726</v>
+        <v>3725</v>
       </c>
       <c r="F1079" t="s">
-        <v>3735</v>
+        <v>3734</v>
       </c>
       <c r="G1079" t="s">
         <v>3703</v>
       </c>
       <c r="H1079" t="s">
-        <v>3736</v>
+        <v>3735</v>
       </c>
       <c r="I1079" t="s">
-        <v>3736</v>
+        <v>3735</v>
       </c>
     </row>
     <row r="1080" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1080" t="s">
-        <v>3737</v>
+        <v>3736</v>
       </c>
       <c r="B1080" t="s">
         <v>66</v>
@@ -44069,24 +44066,24 @@
         <v>3423</v>
       </c>
       <c r="E1080" t="s">
-        <v>3726</v>
+        <v>3725</v>
       </c>
       <c r="F1080" t="s">
-        <v>3738</v>
+        <v>3737</v>
       </c>
       <c r="G1080" t="s">
         <v>3703</v>
       </c>
       <c r="H1080" t="s">
-        <v>3739</v>
+        <v>3738</v>
       </c>
       <c r="I1080" t="s">
-        <v>3739</v>
+        <v>3738</v>
       </c>
     </row>
     <row r="1081" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1081" t="s">
-        <v>3740</v>
+        <v>3739</v>
       </c>
       <c r="B1081" t="s">
         <v>66</v>
@@ -44098,24 +44095,24 @@
         <v>3423</v>
       </c>
       <c r="E1081" t="s">
-        <v>3726</v>
+        <v>3725</v>
       </c>
       <c r="F1081" t="s">
+        <v>3740</v>
+      </c>
+      <c r="G1081" t="s">
+        <v>3729</v>
+      </c>
+      <c r="H1081" t="s">
         <v>3741</v>
       </c>
-      <c r="G1081" t="s">
-        <v>3730</v>
-      </c>
-      <c r="H1081" t="s">
-        <v>3742</v>
-      </c>
       <c r="I1081" t="s">
-        <v>3742</v>
+        <v>3741</v>
       </c>
     </row>
     <row r="1082" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1082" t="s">
-        <v>3743</v>
+        <v>3742</v>
       </c>
       <c r="B1082" t="s">
         <v>66</v>
@@ -44127,7 +44124,7 @@
         <v>3423</v>
       </c>
       <c r="E1082" t="s">
-        <v>3708</v>
+        <v>3743</v>
       </c>
       <c r="F1082" t="s">
         <v>3744</v>
@@ -44139,12 +44136,12 @@
         <v>3745</v>
       </c>
       <c r="I1082" t="s">
-        <v>3746</v>
+        <v>3745</v>
       </c>
     </row>
     <row r="1083" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1083" t="s">
-        <v>3747</v>
+        <v>3746</v>
       </c>
       <c r="B1083" t="s">
         <v>66</v>
@@ -44156,24 +44153,24 @@
         <v>3423</v>
       </c>
       <c r="E1083" t="s">
+        <v>3747</v>
+      </c>
+      <c r="F1083" t="s">
         <v>3748</v>
       </c>
-      <c r="F1083" t="s">
+      <c r="G1083" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1083" t="s">
         <v>3749</v>
       </c>
-      <c r="G1083" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1083" t="s">
-        <v>3750</v>
-      </c>
       <c r="I1083" t="s">
-        <v>3750</v>
+        <v>3749</v>
       </c>
     </row>
     <row r="1084" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1084" t="s">
-        <v>3751</v>
+        <v>3750</v>
       </c>
       <c r="B1084" t="s">
         <v>66</v>
@@ -44185,24 +44182,24 @@
         <v>3423</v>
       </c>
       <c r="E1084" t="s">
-        <v>3748</v>
+        <v>3747</v>
       </c>
       <c r="F1084" t="s">
+        <v>3751</v>
+      </c>
+      <c r="G1084" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1084" t="s">
         <v>3752</v>
       </c>
-      <c r="G1084" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1084" t="s">
-        <v>3753</v>
-      </c>
       <c r="I1084" t="s">
-        <v>3753</v>
+        <v>3752</v>
       </c>
     </row>
     <row r="1085" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1085" t="s">
-        <v>3754</v>
+        <v>3753</v>
       </c>
       <c r="B1085" t="s">
         <v>66</v>
@@ -44214,24 +44211,24 @@
         <v>3423</v>
       </c>
       <c r="E1085" t="s">
-        <v>3748</v>
+        <v>3747</v>
       </c>
       <c r="F1085" t="s">
+        <v>3754</v>
+      </c>
+      <c r="G1085" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1085" t="s">
         <v>3755</v>
       </c>
-      <c r="G1085" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1085" t="s">
-        <v>3756</v>
-      </c>
       <c r="I1085" t="s">
-        <v>3756</v>
+        <v>3755</v>
       </c>
     </row>
     <row r="1086" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1086" t="s">
-        <v>3757</v>
+        <v>3756</v>
       </c>
       <c r="B1086" t="s">
         <v>66</v>
@@ -44243,7 +44240,7 @@
         <v>3423</v>
       </c>
       <c r="E1086" t="s">
-        <v>3708</v>
+        <v>3757</v>
       </c>
       <c r="F1086" t="s">
         <v>3758</v>
@@ -44255,12 +44252,12 @@
         <v>3759</v>
       </c>
       <c r="I1086" t="s">
-        <v>3760</v>
+        <v>3759</v>
       </c>
     </row>
     <row r="1087" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1087" t="s">
-        <v>3761</v>
+        <v>3760</v>
       </c>
       <c r="B1087" t="s">
         <v>66</v>
@@ -44272,10 +44269,10 @@
         <v>3423</v>
       </c>
       <c r="E1087" t="s">
-        <v>3708</v>
+        <v>3761</v>
       </c>
       <c r="F1087" t="s">
-        <v>3727</v>
+        <v>3726</v>
       </c>
       <c r="G1087" t="s">
         <v>10</v>
@@ -44284,12 +44281,12 @@
         <v>3762</v>
       </c>
       <c r="I1087" t="s">
-        <v>3763</v>
+        <v>3762</v>
       </c>
     </row>
     <row r="1088" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1088" t="s">
-        <v>3764</v>
+        <v>3763</v>
       </c>
       <c r="B1088" t="s">
         <v>66</v>
@@ -44301,24 +44298,24 @@
         <v>3423</v>
       </c>
       <c r="E1088" t="s">
-        <v>3708</v>
+        <v>3761</v>
       </c>
       <c r="F1088" t="s">
+        <v>3764</v>
+      </c>
+      <c r="G1088" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1088" t="s">
         <v>3765</v>
       </c>
-      <c r="G1088" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1088" t="s">
-        <v>3766</v>
-      </c>
       <c r="I1088" t="s">
-        <v>3767</v>
+        <v>3765</v>
       </c>
     </row>
     <row r="1089" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1089" t="s">
-        <v>3768</v>
+        <v>3766</v>
       </c>
       <c r="B1089" t="s">
         <v>66</v>
@@ -44330,24 +44327,24 @@
         <v>3423</v>
       </c>
       <c r="E1089" t="s">
-        <v>3708</v>
+        <v>3761</v>
       </c>
       <c r="F1089" t="s">
-        <v>3769</v>
+        <v>3767</v>
       </c>
       <c r="G1089" t="s">
         <v>10</v>
       </c>
       <c r="H1089" t="s">
-        <v>3770</v>
+        <v>3768</v>
       </c>
       <c r="I1089" t="s">
-        <v>3771</v>
+        <v>3768</v>
       </c>
     </row>
     <row r="1090" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1090" t="s">
-        <v>3772</v>
+        <v>3769</v>
       </c>
       <c r="B1090" t="s">
         <v>66</v>
@@ -44359,24 +44356,24 @@
         <v>3423</v>
       </c>
       <c r="E1090" t="s">
-        <v>3708</v>
+        <v>3770</v>
       </c>
       <c r="F1090" t="s">
-        <v>3773</v>
+        <v>3771</v>
       </c>
       <c r="G1090" t="s">
         <v>10</v>
       </c>
       <c r="H1090" t="s">
-        <v>3774</v>
+        <v>3772</v>
       </c>
       <c r="I1090" t="s">
-        <v>3775</v>
+        <v>3772</v>
       </c>
     </row>
     <row r="1091" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1091" t="s">
-        <v>3776</v>
+        <v>3773</v>
       </c>
       <c r="B1091" t="s">
         <v>66</v>
@@ -44388,24 +44385,24 @@
         <v>3423</v>
       </c>
       <c r="E1091" t="s">
-        <v>3708</v>
+        <v>3770</v>
       </c>
       <c r="F1091" t="s">
-        <v>3777</v>
+        <v>3774</v>
       </c>
       <c r="G1091" t="s">
         <v>10</v>
       </c>
       <c r="H1091" t="s">
-        <v>3778</v>
+        <v>3775</v>
       </c>
       <c r="I1091" t="s">
-        <v>3779</v>
+        <v>3775</v>
       </c>
     </row>
     <row r="1092" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1092" t="s">
-        <v>3780</v>
+        <v>3776</v>
       </c>
       <c r="B1092" t="s">
         <v>66</v>
@@ -44417,24 +44414,24 @@
         <v>3423</v>
       </c>
       <c r="E1092" t="s">
-        <v>3781</v>
+        <v>3777</v>
       </c>
       <c r="F1092" t="s">
-        <v>3782</v>
+        <v>3778</v>
       </c>
       <c r="G1092" t="s">
         <v>10</v>
       </c>
       <c r="H1092" t="s">
-        <v>3783</v>
+        <v>3779</v>
       </c>
       <c r="I1092" t="s">
-        <v>3783</v>
+        <v>3779</v>
       </c>
     </row>
     <row r="1093" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1093" t="s">
-        <v>3784</v>
+        <v>3780</v>
       </c>
       <c r="B1093" t="s">
         <v>66</v>
@@ -44446,7 +44443,7 @@
         <v>3423</v>
       </c>
       <c r="E1093" t="s">
-        <v>3785</v>
+        <v>3781</v>
       </c>
       <c r="F1093" t="s">
         <v>3703</v>
@@ -44455,15 +44452,15 @@
         <v>10</v>
       </c>
       <c r="H1093" t="s">
-        <v>3786</v>
+        <v>3782</v>
       </c>
       <c r="I1093" t="s">
-        <v>3786</v>
+        <v>3782</v>
       </c>
     </row>
     <row r="1094" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1094" t="s">
-        <v>3787</v>
+        <v>3783</v>
       </c>
       <c r="B1094" t="s">
         <v>66</v>
@@ -44475,24 +44472,24 @@
         <v>3423</v>
       </c>
       <c r="E1094" t="s">
-        <v>3788</v>
+        <v>3784</v>
       </c>
       <c r="F1094" t="s">
-        <v>3789</v>
+        <v>3785</v>
       </c>
       <c r="G1094" t="s">
         <v>10</v>
       </c>
       <c r="H1094" t="s">
-        <v>3790</v>
+        <v>3786</v>
       </c>
       <c r="I1094" t="s">
-        <v>3790</v>
+        <v>3786</v>
       </c>
     </row>
     <row r="1095" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1095" t="s">
-        <v>3791</v>
+        <v>3787</v>
       </c>
       <c r="B1095" t="s">
         <v>66</v>
@@ -44504,24 +44501,24 @@
         <v>3423</v>
       </c>
       <c r="E1095" t="s">
-        <v>3792</v>
+        <v>3788</v>
       </c>
       <c r="F1095" t="s">
-        <v>3793</v>
+        <v>3789</v>
       </c>
       <c r="G1095" t="s">
         <v>10</v>
       </c>
       <c r="H1095" t="s">
-        <v>3794</v>
+        <v>3790</v>
       </c>
       <c r="I1095" t="s">
-        <v>3794</v>
+        <v>3790</v>
       </c>
     </row>
     <row r="1096" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1096" t="s">
-        <v>3795</v>
+        <v>3791</v>
       </c>
       <c r="B1096" t="s">
         <v>66</v>
@@ -44533,7 +44530,7 @@
         <v>3423</v>
       </c>
       <c r="E1096" t="s">
-        <v>3796</v>
+        <v>3792</v>
       </c>
       <c r="F1096" t="s">
         <v>10</v>
@@ -44542,15 +44539,15 @@
         <v>10</v>
       </c>
       <c r="H1096" t="s">
-        <v>3796</v>
+        <v>3792</v>
       </c>
       <c r="I1096" t="s">
-        <v>3796</v>
+        <v>3792</v>
       </c>
     </row>
     <row r="1097" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1097" t="s">
-        <v>3797</v>
+        <v>3793</v>
       </c>
       <c r="B1097" t="s">
         <v>66</v>
@@ -44562,7 +44559,7 @@
         <v>3423</v>
       </c>
       <c r="E1097" t="s">
-        <v>3798</v>
+        <v>3794</v>
       </c>
       <c r="F1097" t="s">
         <v>10</v>
@@ -44571,15 +44568,15 @@
         <v>10</v>
       </c>
       <c r="H1097" t="s">
-        <v>3798</v>
+        <v>3794</v>
       </c>
       <c r="I1097" t="s">
-        <v>3798</v>
+        <v>3794</v>
       </c>
     </row>
     <row r="1098" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1098" t="s">
-        <v>3799</v>
+        <v>3795</v>
       </c>
       <c r="B1098" t="s">
         <v>66</v>
@@ -44591,24 +44588,24 @@
         <v>3423</v>
       </c>
       <c r="E1098" t="s">
-        <v>3800</v>
+        <v>3796</v>
       </c>
       <c r="F1098" t="s">
-        <v>3801</v>
+        <v>3797</v>
       </c>
       <c r="G1098" t="s">
         <v>10</v>
       </c>
       <c r="H1098" t="s">
-        <v>3802</v>
+        <v>3798</v>
       </c>
       <c r="I1098" t="s">
-        <v>3802</v>
+        <v>3798</v>
       </c>
     </row>
     <row r="1099" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1099" t="s">
-        <v>3803</v>
+        <v>3799</v>
       </c>
       <c r="B1099" t="s">
         <v>66</v>
@@ -44620,24 +44617,24 @@
         <v>3423</v>
       </c>
       <c r="E1099" t="s">
-        <v>3804</v>
+        <v>3796</v>
       </c>
       <c r="F1099" t="s">
-        <v>3805</v>
+        <v>3800</v>
       </c>
       <c r="G1099" t="s">
         <v>10</v>
       </c>
       <c r="H1099" t="s">
-        <v>3806</v>
+        <v>3801</v>
       </c>
       <c r="I1099" t="s">
-        <v>3806</v>
+        <v>3802</v>
       </c>
     </row>
     <row r="1100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1100" t="s">
-        <v>3807</v>
+        <v>3803</v>
       </c>
       <c r="B1100" t="s">
         <v>66</v>
@@ -44649,24 +44646,24 @@
         <v>3423</v>
       </c>
       <c r="E1100" t="s">
-        <v>3808</v>
+        <v>3804</v>
       </c>
       <c r="F1100" t="s">
-        <v>3773</v>
+        <v>3771</v>
       </c>
       <c r="G1100" t="s">
         <v>10</v>
       </c>
       <c r="H1100" t="s">
-        <v>3809</v>
+        <v>3805</v>
       </c>
       <c r="I1100" t="s">
-        <v>3809</v>
+        <v>3805</v>
       </c>
     </row>
     <row r="1101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1101" t="s">
-        <v>3810</v>
+        <v>3806</v>
       </c>
       <c r="B1101" t="s">
         <v>120</v>
@@ -44681,21 +44678,21 @@
         <v>2384</v>
       </c>
       <c r="F1101" t="s">
-        <v>3811</v>
+        <v>3807</v>
       </c>
       <c r="G1101" t="s">
-        <v>3812</v>
+        <v>3808</v>
       </c>
       <c r="H1101" t="s">
-        <v>3813</v>
+        <v>3809</v>
       </c>
       <c r="I1101" t="s">
-        <v>3813</v>
+        <v>3809</v>
       </c>
     </row>
     <row r="1102" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1102" t="s">
-        <v>3814</v>
+        <v>3810</v>
       </c>
       <c r="B1102" t="s">
         <v>120</v>
@@ -44710,21 +44707,21 @@
         <v>2384</v>
       </c>
       <c r="F1102" t="s">
-        <v>3811</v>
+        <v>3807</v>
       </c>
       <c r="G1102" t="s">
         <v>2395</v>
       </c>
       <c r="H1102" t="s">
-        <v>3815</v>
+        <v>3811</v>
       </c>
       <c r="I1102" t="s">
-        <v>3815</v>
+        <v>3811</v>
       </c>
     </row>
     <row r="1103" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1103" t="s">
-        <v>3816</v>
+        <v>3812</v>
       </c>
       <c r="B1103" t="s">
         <v>120</v>
@@ -44742,18 +44739,18 @@
         <v>2385</v>
       </c>
       <c r="G1103" t="s">
-        <v>3817</v>
+        <v>3813</v>
       </c>
       <c r="H1103" t="s">
-        <v>3818</v>
+        <v>3814</v>
       </c>
       <c r="I1103" t="s">
-        <v>3818</v>
+        <v>3814</v>
       </c>
     </row>
     <row r="1104" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1104" t="s">
-        <v>3819</v>
+        <v>3815</v>
       </c>
       <c r="B1104" t="s">
         <v>120</v>
@@ -44774,15 +44771,15 @@
         <v>2398</v>
       </c>
       <c r="H1104" t="s">
-        <v>3820</v>
+        <v>3816</v>
       </c>
       <c r="I1104" t="s">
-        <v>3820</v>
+        <v>3816</v>
       </c>
     </row>
     <row r="1105" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1105" t="s">
-        <v>3821</v>
+        <v>3817</v>
       </c>
       <c r="B1105" t="s">
         <v>120</v>
@@ -44800,18 +44797,18 @@
         <v>3459</v>
       </c>
       <c r="G1105" t="s">
-        <v>3812</v>
+        <v>3808</v>
       </c>
       <c r="H1105" t="s">
-        <v>3822</v>
+        <v>3818</v>
       </c>
       <c r="I1105" t="s">
-        <v>3822</v>
+        <v>3818</v>
       </c>
     </row>
     <row r="1106" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1106" t="s">
-        <v>3823</v>
+        <v>3819</v>
       </c>
       <c r="B1106" t="s">
         <v>120</v>
@@ -44826,21 +44823,21 @@
         <v>2384</v>
       </c>
       <c r="F1106" t="s">
-        <v>3824</v>
+        <v>3820</v>
       </c>
       <c r="G1106" t="s">
         <v>2389</v>
       </c>
       <c r="H1106" t="s">
-        <v>3825</v>
+        <v>3821</v>
       </c>
       <c r="I1106" t="s">
-        <v>3825</v>
+        <v>3821</v>
       </c>
     </row>
     <row r="1107" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1107" t="s">
-        <v>3826</v>
+        <v>3822</v>
       </c>
       <c r="B1107" t="s">
         <v>120</v>
@@ -44855,21 +44852,21 @@
         <v>2384</v>
       </c>
       <c r="F1107" t="s">
-        <v>3811</v>
+        <v>3807</v>
       </c>
       <c r="G1107" t="s">
         <v>2392</v>
       </c>
       <c r="H1107" t="s">
-        <v>3827</v>
+        <v>3823</v>
       </c>
       <c r="I1107" t="s">
-        <v>3827</v>
+        <v>3823</v>
       </c>
     </row>
     <row r="1108" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1108" t="s">
-        <v>3828</v>
+        <v>3824</v>
       </c>
       <c r="B1108" t="s">
         <v>120</v>
@@ -44887,18 +44884,18 @@
         <v>2385</v>
       </c>
       <c r="G1108" t="s">
-        <v>3829</v>
+        <v>3825</v>
       </c>
       <c r="H1108" t="s">
-        <v>3830</v>
+        <v>3826</v>
       </c>
       <c r="I1108" t="s">
-        <v>3830</v>
+        <v>3826</v>
       </c>
     </row>
     <row r="1109" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1109" t="s">
-        <v>3831</v>
+        <v>3827</v>
       </c>
       <c r="B1109" t="s">
         <v>120</v>
@@ -44913,21 +44910,21 @@
         <v>2384</v>
       </c>
       <c r="F1109" t="s">
-        <v>3824</v>
+        <v>3820</v>
       </c>
       <c r="G1109" t="s">
-        <v>3829</v>
+        <v>3825</v>
       </c>
       <c r="H1109" t="s">
-        <v>3832</v>
+        <v>3828</v>
       </c>
       <c r="I1109" t="s">
-        <v>3832</v>
+        <v>3828</v>
       </c>
     </row>
     <row r="1110" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1110" t="s">
-        <v>3833</v>
+        <v>3829</v>
       </c>
       <c r="B1110" t="s">
         <v>120</v>
@@ -44945,18 +44942,18 @@
         <v>2385</v>
       </c>
       <c r="G1110" t="s">
-        <v>3834</v>
+        <v>3830</v>
       </c>
       <c r="H1110" t="s">
-        <v>3835</v>
+        <v>3831</v>
       </c>
       <c r="I1110" t="s">
-        <v>3835</v>
+        <v>3831</v>
       </c>
     </row>
     <row r="1111" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1111" t="s">
-        <v>3836</v>
+        <v>3832</v>
       </c>
       <c r="B1111" t="s">
         <v>120</v>
@@ -44971,21 +44968,21 @@
         <v>2384</v>
       </c>
       <c r="F1111" t="s">
-        <v>3824</v>
+        <v>3820</v>
       </c>
       <c r="G1111" t="s">
-        <v>3812</v>
+        <v>3808</v>
       </c>
       <c r="H1111" t="s">
-        <v>3837</v>
+        <v>3833</v>
       </c>
       <c r="I1111" t="s">
-        <v>3837</v>
+        <v>3833</v>
       </c>
     </row>
     <row r="1112" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1112" t="s">
-        <v>3838</v>
+        <v>3834</v>
       </c>
       <c r="B1112" t="s">
         <v>120</v>
@@ -45000,21 +44997,21 @@
         <v>2384</v>
       </c>
       <c r="F1112" t="s">
-        <v>3811</v>
+        <v>3807</v>
       </c>
       <c r="G1112" t="s">
         <v>2389</v>
       </c>
       <c r="H1112" t="s">
-        <v>3839</v>
+        <v>3835</v>
       </c>
       <c r="I1112" t="s">
-        <v>3839</v>
+        <v>3835</v>
       </c>
     </row>
     <row r="1113" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1113" t="s">
-        <v>3840</v>
+        <v>3836</v>
       </c>
       <c r="B1113" t="s">
         <v>120</v>
@@ -45029,21 +45026,21 @@
         <v>2384</v>
       </c>
       <c r="F1113" t="s">
-        <v>3824</v>
+        <v>3820</v>
       </c>
       <c r="G1113" t="s">
-        <v>3834</v>
+        <v>3830</v>
       </c>
       <c r="H1113" t="s">
-        <v>3841</v>
+        <v>3837</v>
       </c>
       <c r="I1113" t="s">
-        <v>3841</v>
+        <v>3837</v>
       </c>
     </row>
     <row r="1114" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1114" t="s">
-        <v>3842</v>
+        <v>3838</v>
       </c>
       <c r="B1114" t="s">
         <v>120</v>
@@ -45058,21 +45055,21 @@
         <v>2384</v>
       </c>
       <c r="F1114" t="s">
-        <v>3811</v>
+        <v>3807</v>
       </c>
       <c r="G1114" t="s">
         <v>2386</v>
       </c>
       <c r="H1114" t="s">
-        <v>3843</v>
+        <v>3839</v>
       </c>
       <c r="I1114" t="s">
-        <v>3843</v>
+        <v>3839</v>
       </c>
     </row>
     <row r="1115" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1115" t="s">
-        <v>3844</v>
+        <v>3840</v>
       </c>
       <c r="B1115" t="s">
         <v>120</v>
@@ -45087,21 +45084,21 @@
         <v>2384</v>
       </c>
       <c r="F1115" t="s">
-        <v>3824</v>
+        <v>3820</v>
       </c>
       <c r="G1115" t="s">
         <v>2392</v>
       </c>
       <c r="H1115" t="s">
-        <v>3845</v>
+        <v>3841</v>
       </c>
       <c r="I1115" t="s">
-        <v>3845</v>
+        <v>3841</v>
       </c>
     </row>
     <row r="1116" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1116" t="s">
-        <v>3846</v>
+        <v>3842</v>
       </c>
       <c r="B1116" t="s">
         <v>120</v>
@@ -45122,15 +45119,15 @@
         <v>2389</v>
       </c>
       <c r="H1116" t="s">
-        <v>3847</v>
+        <v>3843</v>
       </c>
       <c r="I1116" t="s">
-        <v>3847</v>
+        <v>3843</v>
       </c>
     </row>
     <row r="1117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1117" t="s">
-        <v>3848</v>
+        <v>3844</v>
       </c>
       <c r="B1117" t="s">
         <v>120</v>
@@ -45145,21 +45142,21 @@
         <v>2384</v>
       </c>
       <c r="F1117" t="s">
-        <v>3824</v>
+        <v>3820</v>
       </c>
       <c r="G1117" t="s">
-        <v>3817</v>
+        <v>3813</v>
       </c>
       <c r="H1117" t="s">
-        <v>3849</v>
+        <v>3845</v>
       </c>
       <c r="I1117" t="s">
-        <v>3849</v>
+        <v>3845</v>
       </c>
     </row>
     <row r="1118" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1118" t="s">
-        <v>3850</v>
+        <v>3846</v>
       </c>
       <c r="B1118" t="s">
         <v>120</v>
@@ -45180,15 +45177,15 @@
         <v>2398</v>
       </c>
       <c r="H1118" t="s">
-        <v>3820</v>
+        <v>3816</v>
       </c>
       <c r="I1118" t="s">
-        <v>3820</v>
+        <v>3816</v>
       </c>
     </row>
     <row r="1119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1119" t="s">
-        <v>3851</v>
+        <v>3847</v>
       </c>
       <c r="B1119" t="s">
         <v>120</v>
@@ -45209,15 +45206,15 @@
         <v>2392</v>
       </c>
       <c r="H1119" t="s">
-        <v>3852</v>
+        <v>3848</v>
       </c>
       <c r="I1119" t="s">
-        <v>3852</v>
+        <v>3848</v>
       </c>
     </row>
     <row r="1120" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1120" t="s">
-        <v>3853</v>
+        <v>3849</v>
       </c>
       <c r="B1120" t="s">
         <v>120</v>
@@ -45232,21 +45229,21 @@
         <v>2384</v>
       </c>
       <c r="F1120" t="s">
-        <v>3811</v>
+        <v>3807</v>
       </c>
       <c r="G1120" t="s">
-        <v>3834</v>
+        <v>3830</v>
       </c>
       <c r="H1120" t="s">
-        <v>3854</v>
+        <v>3850</v>
       </c>
       <c r="I1120" t="s">
-        <v>3854</v>
+        <v>3850</v>
       </c>
     </row>
     <row r="1121" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1121" t="s">
-        <v>3855</v>
+        <v>3851</v>
       </c>
       <c r="B1121" t="s">
         <v>120</v>
@@ -45261,21 +45258,21 @@
         <v>2384</v>
       </c>
       <c r="F1121" t="s">
-        <v>3824</v>
+        <v>3820</v>
       </c>
       <c r="G1121" t="s">
         <v>2386</v>
       </c>
       <c r="H1121" t="s">
-        <v>3856</v>
+        <v>3852</v>
       </c>
       <c r="I1121" t="s">
-        <v>3856</v>
+        <v>3852</v>
       </c>
     </row>
     <row r="1122" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1122" t="s">
-        <v>3857</v>
+        <v>3853</v>
       </c>
       <c r="B1122" t="s">
         <v>120</v>
@@ -45293,18 +45290,18 @@
         <v>3459</v>
       </c>
       <c r="G1122" t="s">
-        <v>3834</v>
+        <v>3830</v>
       </c>
       <c r="H1122" t="s">
-        <v>3858</v>
+        <v>3854</v>
       </c>
       <c r="I1122" t="s">
-        <v>3858</v>
+        <v>3854</v>
       </c>
     </row>
     <row r="1123" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1123" t="s">
-        <v>3859</v>
+        <v>3855</v>
       </c>
       <c r="B1123" t="s">
         <v>120</v>
@@ -45325,15 +45322,15 @@
         <v>2395</v>
       </c>
       <c r="H1123" t="s">
-        <v>3860</v>
+        <v>3856</v>
       </c>
       <c r="I1123" t="s">
-        <v>3860</v>
+        <v>3856</v>
       </c>
     </row>
     <row r="1124" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1124" t="s">
-        <v>3861</v>
+        <v>3857</v>
       </c>
       <c r="B1124" t="s">
         <v>120</v>
@@ -45351,18 +45348,18 @@
         <v>2385</v>
       </c>
       <c r="G1124" t="s">
-        <v>3812</v>
+        <v>3808</v>
       </c>
       <c r="H1124" t="s">
-        <v>3862</v>
+        <v>3858</v>
       </c>
       <c r="I1124" t="s">
-        <v>3862</v>
+        <v>3858</v>
       </c>
     </row>
     <row r="1125" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1125" t="s">
-        <v>3863</v>
+        <v>3859</v>
       </c>
       <c r="B1125" t="s">
         <v>120</v>
@@ -45377,21 +45374,21 @@
         <v>2384</v>
       </c>
       <c r="F1125" t="s">
-        <v>3824</v>
+        <v>3820</v>
       </c>
       <c r="G1125" t="s">
         <v>2395</v>
       </c>
       <c r="H1125" t="s">
-        <v>3864</v>
+        <v>3860</v>
       </c>
       <c r="I1125" t="s">
-        <v>3864</v>
+        <v>3860</v>
       </c>
     </row>
     <row r="1126" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1126" t="s">
-        <v>3865</v>
+        <v>3861</v>
       </c>
       <c r="B1126" t="s">
         <v>120</v>
@@ -45412,15 +45409,15 @@
         <v>2386</v>
       </c>
       <c r="H1126" t="s">
-        <v>3866</v>
+        <v>3862</v>
       </c>
       <c r="I1126" t="s">
-        <v>3866</v>
+        <v>3862</v>
       </c>
     </row>
     <row r="1127" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1127" t="s">
-        <v>3867</v>
+        <v>3863</v>
       </c>
       <c r="B1127" t="s">
         <v>120</v>
@@ -45435,21 +45432,21 @@
         <v>2384</v>
       </c>
       <c r="F1127" t="s">
-        <v>3824</v>
+        <v>3820</v>
       </c>
       <c r="G1127" t="s">
         <v>2398</v>
       </c>
       <c r="H1127" t="s">
-        <v>3868</v>
+        <v>3864</v>
       </c>
       <c r="I1127" t="s">
-        <v>3868</v>
+        <v>3864</v>
       </c>
     </row>
     <row r="1128" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1128" t="s">
-        <v>3869</v>
+        <v>3865</v>
       </c>
       <c r="B1128" t="s">
         <v>66</v>
@@ -45461,7 +45458,7 @@
         <v>3423</v>
       </c>
       <c r="E1128" t="s">
-        <v>3870</v>
+        <v>3866</v>
       </c>
       <c r="F1128" t="s">
         <v>10</v>
@@ -45470,15 +45467,15 @@
         <v>10</v>
       </c>
       <c r="H1128" t="s">
-        <v>3870</v>
+        <v>3866</v>
       </c>
       <c r="I1128" t="s">
-        <v>3871</v>
+        <v>3867</v>
       </c>
     </row>
     <row r="1129" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1129" t="s">
-        <v>3872</v>
+        <v>3868</v>
       </c>
       <c r="B1129" t="s">
         <v>14</v>
@@ -45499,15 +45496,15 @@
         <v>10</v>
       </c>
       <c r="H1129" t="s">
-        <v>3873</v>
+        <v>3869</v>
       </c>
       <c r="I1129" t="s">
-        <v>3873</v>
+        <v>3869</v>
       </c>
     </row>
     <row r="1130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1130" t="s">
-        <v>3874</v>
+        <v>3870</v>
       </c>
       <c r="B1130" t="s">
         <v>14</v>
@@ -45522,21 +45519,21 @@
         <v>553</v>
       </c>
       <c r="F1130" t="s">
-        <v>3875</v>
+        <v>3871</v>
       </c>
       <c r="G1130" t="s">
         <v>10</v>
       </c>
       <c r="H1130" t="s">
-        <v>3876</v>
+        <v>3872</v>
       </c>
       <c r="I1130" t="s">
-        <v>3877</v>
+        <v>3873</v>
       </c>
     </row>
     <row r="1131" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1131" t="s">
-        <v>3878</v>
+        <v>3874</v>
       </c>
       <c r="B1131" t="s">
         <v>14</v>
@@ -45551,21 +45548,21 @@
         <v>553</v>
       </c>
       <c r="F1131" t="s">
+        <v>3871</v>
+      </c>
+      <c r="G1131" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1131" t="s">
+        <v>3872</v>
+      </c>
+      <c r="I1131" t="s">
         <v>3875</v>
-      </c>
-      <c r="G1131" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1131" t="s">
-        <v>3876</v>
-      </c>
-      <c r="I1131" t="s">
-        <v>3879</v>
       </c>
     </row>
     <row r="1132" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1132" t="s">
-        <v>3880</v>
+        <v>3876</v>
       </c>
       <c r="B1132" t="s">
         <v>14</v>
@@ -45586,15 +45583,15 @@
         <v>10</v>
       </c>
       <c r="H1132" t="s">
-        <v>3881</v>
+        <v>3877</v>
       </c>
       <c r="I1132" t="s">
-        <v>3881</v>
+        <v>3877</v>
       </c>
     </row>
     <row r="1133" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1133" t="s">
-        <v>3882</v>
+        <v>3878</v>
       </c>
       <c r="B1133" t="s">
         <v>14</v>
@@ -45609,21 +45606,21 @@
         <v>553</v>
       </c>
       <c r="F1133" t="s">
-        <v>3875</v>
+        <v>3871</v>
       </c>
       <c r="G1133" t="s">
         <v>10</v>
       </c>
       <c r="H1133" t="s">
-        <v>3876</v>
+        <v>3872</v>
       </c>
       <c r="I1133" t="s">
-        <v>3883</v>
+        <v>3879</v>
       </c>
     </row>
     <row r="1134" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1134" t="s">
-        <v>3884</v>
+        <v>3880</v>
       </c>
       <c r="B1134" t="s">
         <v>66</v>
@@ -45635,24 +45632,24 @@
         <v>3423</v>
       </c>
       <c r="E1134" t="s">
-        <v>3885</v>
+        <v>3881</v>
       </c>
       <c r="F1134" t="s">
-        <v>3886</v>
+        <v>3882</v>
       </c>
       <c r="G1134" t="s">
         <v>10</v>
       </c>
       <c r="H1134" t="s">
-        <v>3887</v>
+        <v>3883</v>
       </c>
       <c r="I1134" t="s">
-        <v>3887</v>
+        <v>3883</v>
       </c>
     </row>
     <row r="1135" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1135" t="s">
-        <v>3888</v>
+        <v>3884</v>
       </c>
       <c r="B1135" t="s">
         <v>66</v>
@@ -45664,7 +45661,7 @@
         <v>3423</v>
       </c>
       <c r="E1135" t="s">
-        <v>3885</v>
+        <v>3881</v>
       </c>
       <c r="F1135" t="s">
         <v>3267</v>
@@ -45673,15 +45670,15 @@
         <v>10</v>
       </c>
       <c r="H1135" t="s">
-        <v>3889</v>
+        <v>3885</v>
       </c>
       <c r="I1135" t="s">
-        <v>3889</v>
+        <v>3885</v>
       </c>
     </row>
     <row r="1136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1136" t="s">
-        <v>3890</v>
+        <v>3886</v>
       </c>
       <c r="B1136" t="s">
         <v>66</v>
@@ -45693,7 +45690,7 @@
         <v>3423</v>
       </c>
       <c r="E1136" t="s">
-        <v>3891</v>
+        <v>3887</v>
       </c>
       <c r="F1136" t="s">
         <v>10</v>
@@ -45702,15 +45699,15 @@
         <v>10</v>
       </c>
       <c r="H1136" t="s">
-        <v>3891</v>
+        <v>3887</v>
       </c>
       <c r="I1136" t="s">
-        <v>3892</v>
+        <v>3888</v>
       </c>
     </row>
     <row r="1137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1137" t="s">
-        <v>3893</v>
+        <v>3889</v>
       </c>
       <c r="B1137" t="s">
         <v>66</v>
@@ -45722,24 +45719,24 @@
         <v>3423</v>
       </c>
       <c r="E1137" t="s">
-        <v>3894</v>
+        <v>3890</v>
       </c>
       <c r="F1137" t="s">
-        <v>3895</v>
+        <v>3891</v>
       </c>
       <c r="G1137" t="s">
         <v>3524</v>
       </c>
       <c r="H1137" t="s">
-        <v>3896</v>
+        <v>3892</v>
       </c>
       <c r="I1137" t="s">
-        <v>3896</v>
+        <v>3892</v>
       </c>
     </row>
     <row r="1138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1138" t="s">
-        <v>3897</v>
+        <v>3893</v>
       </c>
       <c r="B1138" t="s">
         <v>66</v>
@@ -45751,24 +45748,24 @@
         <v>3423</v>
       </c>
       <c r="E1138" t="s">
+        <v>3890</v>
+      </c>
+      <c r="F1138" t="s">
+        <v>3891</v>
+      </c>
+      <c r="G1138" t="s">
         <v>3894</v>
       </c>
-      <c r="F1138" t="s">
+      <c r="H1138" t="s">
         <v>3895</v>
       </c>
-      <c r="G1138" t="s">
-        <v>3898</v>
-      </c>
-      <c r="H1138" t="s">
-        <v>3899</v>
-      </c>
       <c r="I1138" t="s">
-        <v>3899</v>
+        <v>3895</v>
       </c>
     </row>
     <row r="1139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1139" t="s">
-        <v>3900</v>
+        <v>3896</v>
       </c>
       <c r="B1139" t="s">
         <v>66</v>
@@ -45780,7 +45777,7 @@
         <v>3423</v>
       </c>
       <c r="E1139" t="s">
-        <v>3901</v>
+        <v>3897</v>
       </c>
       <c r="F1139" t="s">
         <v>10</v>
@@ -45789,15 +45786,15 @@
         <v>10</v>
       </c>
       <c r="H1139" t="s">
-        <v>3901</v>
+        <v>3897</v>
       </c>
       <c r="I1139" t="s">
-        <v>3901</v>
+        <v>3897</v>
       </c>
     </row>
     <row r="1140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1140" t="s">
-        <v>3902</v>
+        <v>3898</v>
       </c>
       <c r="B1140" t="s">
         <v>66</v>
@@ -45809,24 +45806,24 @@
         <v>3423</v>
       </c>
       <c r="E1140" t="s">
-        <v>3903</v>
+        <v>3899</v>
       </c>
       <c r="F1140" t="s">
-        <v>3904</v>
+        <v>3900</v>
       </c>
       <c r="G1140" t="s">
         <v>10</v>
       </c>
       <c r="H1140" t="s">
-        <v>3905</v>
+        <v>3901</v>
       </c>
       <c r="I1140" t="s">
-        <v>3905</v>
+        <v>3901</v>
       </c>
     </row>
     <row r="1141" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1141" t="s">
-        <v>3906</v>
+        <v>3902</v>
       </c>
       <c r="B1141" t="s">
         <v>66</v>
@@ -45838,24 +45835,24 @@
         <v>3423</v>
       </c>
       <c r="E1141" t="s">
+        <v>3899</v>
+      </c>
+      <c r="F1141" t="s">
         <v>3903</v>
       </c>
-      <c r="F1141" t="s">
-        <v>3907</v>
-      </c>
       <c r="G1141" t="s">
         <v>10</v>
       </c>
       <c r="H1141" t="s">
-        <v>3908</v>
+        <v>3904</v>
       </c>
       <c r="I1141" t="s">
-        <v>3908</v>
+        <v>3904</v>
       </c>
     </row>
     <row r="1142" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1142" t="s">
-        <v>3909</v>
+        <v>3905</v>
       </c>
       <c r="B1142" t="s">
         <v>66</v>
@@ -45867,24 +45864,24 @@
         <v>3423</v>
       </c>
       <c r="E1142" t="s">
-        <v>3903</v>
+        <v>3899</v>
       </c>
       <c r="F1142" t="s">
-        <v>3910</v>
+        <v>3906</v>
       </c>
       <c r="G1142" t="s">
         <v>10</v>
       </c>
       <c r="H1142" t="s">
-        <v>3911</v>
+        <v>3907</v>
       </c>
       <c r="I1142" t="s">
-        <v>3911</v>
+        <v>3907</v>
       </c>
     </row>
     <row r="1143" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1143" t="s">
-        <v>3912</v>
+        <v>3908</v>
       </c>
       <c r="B1143" t="s">
         <v>66</v>
@@ -45896,24 +45893,24 @@
         <v>3423</v>
       </c>
       <c r="E1143" t="s">
-        <v>3913</v>
+        <v>3909</v>
       </c>
       <c r="F1143" t="s">
-        <v>3914</v>
+        <v>3910</v>
       </c>
       <c r="G1143" t="s">
         <v>10</v>
       </c>
       <c r="H1143" t="s">
-        <v>3915</v>
+        <v>3911</v>
       </c>
       <c r="I1143" t="s">
-        <v>3913</v>
+        <v>3912</v>
       </c>
     </row>
     <row r="1144" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1144" t="s">
-        <v>3916</v>
+        <v>3913</v>
       </c>
       <c r="B1144" t="s">
         <v>66</v>
@@ -45925,24 +45922,24 @@
         <v>3423</v>
       </c>
       <c r="E1144" t="s">
-        <v>3917</v>
+        <v>3909</v>
       </c>
       <c r="F1144" t="s">
-        <v>3918</v>
+        <v>3914</v>
       </c>
       <c r="G1144" t="s">
         <v>10</v>
       </c>
       <c r="H1144" t="s">
-        <v>3919</v>
+        <v>3915</v>
       </c>
       <c r="I1144" t="s">
-        <v>3920</v>
+        <v>3916</v>
       </c>
     </row>
     <row r="1145" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1145" t="s">
-        <v>3921</v>
+        <v>3917</v>
       </c>
       <c r="B1145" t="s">
         <v>66</v>
@@ -45954,24 +45951,24 @@
         <v>3423</v>
       </c>
       <c r="E1145" t="s">
-        <v>3922</v>
+        <v>3918</v>
       </c>
       <c r="F1145" t="s">
-        <v>3923</v>
+        <v>3919</v>
       </c>
       <c r="G1145" t="s">
-        <v>3924</v>
+        <v>3920</v>
       </c>
       <c r="H1145" t="s">
-        <v>3925</v>
+        <v>3921</v>
       </c>
       <c r="I1145" t="s">
-        <v>3925</v>
+        <v>3921</v>
       </c>
     </row>
     <row r="1146" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1146" t="s">
-        <v>3926</v>
+        <v>3922</v>
       </c>
       <c r="B1146" t="s">
         <v>66</v>
@@ -45983,24 +45980,24 @@
         <v>3423</v>
       </c>
       <c r="E1146" t="s">
-        <v>3922</v>
+        <v>3918</v>
       </c>
       <c r="F1146" t="s">
-        <v>3927</v>
+        <v>3923</v>
       </c>
       <c r="G1146" t="s">
         <v>462</v>
       </c>
       <c r="H1146" t="s">
-        <v>3928</v>
+        <v>3924</v>
       </c>
       <c r="I1146" t="s">
-        <v>3928</v>
+        <v>3924</v>
       </c>
     </row>
     <row r="1147" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1147" t="s">
-        <v>3929</v>
+        <v>3925</v>
       </c>
       <c r="B1147" t="s">
         <v>66</v>
@@ -46012,24 +46009,24 @@
         <v>3423</v>
       </c>
       <c r="E1147" t="s">
-        <v>3922</v>
+        <v>3918</v>
       </c>
       <c r="F1147" t="s">
-        <v>3923</v>
+        <v>3919</v>
       </c>
       <c r="G1147" t="s">
         <v>504</v>
       </c>
       <c r="H1147" t="s">
-        <v>3930</v>
+        <v>3926</v>
       </c>
       <c r="I1147" t="s">
-        <v>3930</v>
+        <v>3926</v>
       </c>
     </row>
     <row r="1148" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1148" t="s">
-        <v>3931</v>
+        <v>3927</v>
       </c>
       <c r="B1148" t="s">
         <v>66</v>
@@ -46041,24 +46038,24 @@
         <v>3423</v>
       </c>
       <c r="E1148" t="s">
-        <v>3922</v>
+        <v>3918</v>
       </c>
       <c r="F1148" t="s">
-        <v>3927</v>
+        <v>3923</v>
       </c>
       <c r="G1148" t="s">
-        <v>3932</v>
+        <v>3928</v>
       </c>
       <c r="H1148" t="s">
-        <v>3933</v>
+        <v>3929</v>
       </c>
       <c r="I1148" t="s">
-        <v>3933</v>
+        <v>3929</v>
       </c>
     </row>
     <row r="1149" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1149" t="s">
-        <v>3934</v>
+        <v>3930</v>
       </c>
       <c r="B1149" t="s">
         <v>66</v>
@@ -46070,24 +46067,24 @@
         <v>3423</v>
       </c>
       <c r="E1149" t="s">
-        <v>3922</v>
+        <v>3918</v>
       </c>
       <c r="F1149" t="s">
-        <v>3923</v>
+        <v>3919</v>
       </c>
       <c r="G1149" t="s">
         <v>456</v>
       </c>
       <c r="H1149" t="s">
-        <v>3935</v>
+        <v>3931</v>
       </c>
       <c r="I1149" t="s">
-        <v>3935</v>
+        <v>3931</v>
       </c>
     </row>
     <row r="1150" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1150" t="s">
-        <v>3936</v>
+        <v>3932</v>
       </c>
       <c r="B1150" t="s">
         <v>66</v>
@@ -46099,24 +46096,24 @@
         <v>3423</v>
       </c>
       <c r="E1150" t="s">
-        <v>3922</v>
+        <v>3918</v>
       </c>
       <c r="F1150" t="s">
-        <v>3927</v>
+        <v>3923</v>
       </c>
       <c r="G1150" t="s">
-        <v>3937</v>
+        <v>3933</v>
       </c>
       <c r="H1150" t="s">
-        <v>3938</v>
+        <v>3934</v>
       </c>
       <c r="I1150" t="s">
-        <v>3938</v>
+        <v>3934</v>
       </c>
     </row>
     <row r="1151" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1151" t="s">
-        <v>3939</v>
+        <v>3935</v>
       </c>
       <c r="B1151" t="s">
         <v>66</v>
@@ -46128,7 +46125,7 @@
         <v>3423</v>
       </c>
       <c r="E1151" t="s">
-        <v>3940</v>
+        <v>3936</v>
       </c>
       <c r="F1151" t="s">
         <v>10</v>
@@ -46137,15 +46134,15 @@
         <v>10</v>
       </c>
       <c r="H1151" t="s">
-        <v>3940</v>
+        <v>3936</v>
       </c>
       <c r="I1151" t="s">
-        <v>3941</v>
+        <v>3937</v>
       </c>
     </row>
     <row r="1152" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1152" t="s">
-        <v>3942</v>
+        <v>3938</v>
       </c>
       <c r="B1152" t="s">
         <v>66</v>
@@ -46157,7 +46154,7 @@
         <v>3423</v>
       </c>
       <c r="E1152" t="s">
-        <v>3943</v>
+        <v>3939</v>
       </c>
       <c r="F1152" t="s">
         <v>10</v>
@@ -46166,15 +46163,15 @@
         <v>10</v>
       </c>
       <c r="H1152" t="s">
-        <v>3943</v>
+        <v>3939</v>
       </c>
       <c r="I1152" t="s">
-        <v>3943</v>
+        <v>3939</v>
       </c>
     </row>
     <row r="1153" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1153" t="s">
-        <v>3944</v>
+        <v>3940</v>
       </c>
       <c r="B1153" t="s">
         <v>66</v>
@@ -46186,7 +46183,7 @@
         <v>3423</v>
       </c>
       <c r="E1153" t="s">
-        <v>3945</v>
+        <v>3941</v>
       </c>
       <c r="F1153" t="s">
         <v>10</v>
@@ -46195,15 +46192,15 @@
         <v>10</v>
       </c>
       <c r="H1153" t="s">
-        <v>3945</v>
+        <v>3941</v>
       </c>
       <c r="I1153" t="s">
-        <v>3945</v>
+        <v>3941</v>
       </c>
     </row>
     <row r="1154" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1154" t="s">
-        <v>3946</v>
+        <v>3942</v>
       </c>
       <c r="B1154" t="s">
         <v>66</v>
@@ -46215,7 +46212,7 @@
         <v>3423</v>
       </c>
       <c r="E1154" t="s">
-        <v>3947</v>
+        <v>3943</v>
       </c>
       <c r="F1154" t="s">
         <v>10</v>
@@ -46224,15 +46221,15 @@
         <v>10</v>
       </c>
       <c r="H1154" t="s">
-        <v>3947</v>
+        <v>3943</v>
       </c>
       <c r="I1154" t="s">
-        <v>3947</v>
+        <v>3943</v>
       </c>
     </row>
     <row r="1155" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1155" t="s">
-        <v>3948</v>
+        <v>3944</v>
       </c>
       <c r="B1155" t="s">
         <v>120</v>
@@ -46244,7 +46241,7 @@
         <v>3423</v>
       </c>
       <c r="E1155" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="F1155" t="s">
         <v>10</v>
@@ -46253,15 +46250,15 @@
         <v>10</v>
       </c>
       <c r="H1155" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="I1155" t="s">
-        <v>3950</v>
+        <v>3946</v>
       </c>
     </row>
     <row r="1156" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1156" t="s">
-        <v>3951</v>
+        <v>3947</v>
       </c>
       <c r="B1156" t="s">
         <v>120</v>
@@ -46273,7 +46270,7 @@
         <v>3423</v>
       </c>
       <c r="E1156" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="F1156" t="s">
         <v>10</v>
@@ -46282,15 +46279,15 @@
         <v>10</v>
       </c>
       <c r="H1156" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="I1156" t="s">
-        <v>3952</v>
+        <v>3948</v>
       </c>
     </row>
     <row r="1157" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1157" t="s">
-        <v>3953</v>
+        <v>3949</v>
       </c>
       <c r="B1157" t="s">
         <v>120</v>
@@ -46302,7 +46299,7 @@
         <v>3423</v>
       </c>
       <c r="E1157" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="F1157" t="s">
         <v>10</v>
@@ -46311,15 +46308,15 @@
         <v>10</v>
       </c>
       <c r="H1157" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="I1157" t="s">
-        <v>3954</v>
+        <v>3950</v>
       </c>
     </row>
     <row r="1158" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1158" t="s">
-        <v>3955</v>
+        <v>3951</v>
       </c>
       <c r="B1158" t="s">
         <v>120</v>
@@ -46331,7 +46328,7 @@
         <v>3423</v>
       </c>
       <c r="E1158" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="F1158" t="s">
         <v>10</v>
@@ -46340,15 +46337,15 @@
         <v>10</v>
       </c>
       <c r="H1158" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="I1158" t="s">
-        <v>3956</v>
+        <v>3952</v>
       </c>
     </row>
     <row r="1159" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1159" t="s">
-        <v>3957</v>
+        <v>3953</v>
       </c>
       <c r="B1159" t="s">
         <v>120</v>
@@ -46360,7 +46357,7 @@
         <v>3423</v>
       </c>
       <c r="E1159" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="F1159" t="s">
         <v>10</v>
@@ -46369,15 +46366,15 @@
         <v>10</v>
       </c>
       <c r="H1159" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="I1159" t="s">
-        <v>3958</v>
+        <v>3954</v>
       </c>
     </row>
     <row r="1160" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1160" t="s">
-        <v>3959</v>
+        <v>3955</v>
       </c>
       <c r="B1160" t="s">
         <v>120</v>
@@ -46389,7 +46386,7 @@
         <v>3423</v>
       </c>
       <c r="E1160" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="F1160" t="s">
         <v>10</v>
@@ -46398,15 +46395,15 @@
         <v>10</v>
       </c>
       <c r="H1160" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="I1160" t="s">
-        <v>3960</v>
+        <v>3956</v>
       </c>
     </row>
     <row r="1161" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1161" t="s">
-        <v>3961</v>
+        <v>3957</v>
       </c>
       <c r="B1161" t="s">
         <v>120</v>
@@ -46418,7 +46415,7 @@
         <v>3423</v>
       </c>
       <c r="E1161" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="F1161" t="s">
         <v>10</v>
@@ -46427,15 +46424,15 @@
         <v>10</v>
       </c>
       <c r="H1161" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="I1161" t="s">
-        <v>3962</v>
+        <v>3958</v>
       </c>
     </row>
     <row r="1162" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1162" t="s">
-        <v>3963</v>
+        <v>3959</v>
       </c>
       <c r="B1162" t="s">
         <v>120</v>
@@ -46447,7 +46444,7 @@
         <v>3423</v>
       </c>
       <c r="E1162" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="F1162" t="s">
         <v>10</v>
@@ -46456,15 +46453,15 @@
         <v>10</v>
       </c>
       <c r="H1162" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="I1162" t="s">
-        <v>3964</v>
+        <v>3960</v>
       </c>
     </row>
     <row r="1163" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1163" t="s">
-        <v>3965</v>
+        <v>3961</v>
       </c>
       <c r="B1163" t="s">
         <v>120</v>
@@ -46476,7 +46473,7 @@
         <v>3423</v>
       </c>
       <c r="E1163" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="F1163" t="s">
         <v>10</v>
@@ -46485,15 +46482,15 @@
         <v>10</v>
       </c>
       <c r="H1163" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="I1163" t="s">
-        <v>3966</v>
+        <v>3962</v>
       </c>
     </row>
     <row r="1164" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1164" t="s">
-        <v>3967</v>
+        <v>3963</v>
       </c>
       <c r="B1164" t="s">
         <v>120</v>
@@ -46505,7 +46502,7 @@
         <v>3423</v>
       </c>
       <c r="E1164" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="F1164" t="s">
         <v>10</v>
@@ -46514,15 +46511,15 @@
         <v>10</v>
       </c>
       <c r="H1164" t="s">
-        <v>3949</v>
+        <v>3945</v>
       </c>
       <c r="I1164" t="s">
-        <v>3968</v>
+        <v>3964</v>
       </c>
     </row>
     <row r="1165" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1165" t="s">
-        <v>3969</v>
+        <v>3965</v>
       </c>
       <c r="B1165" t="s">
         <v>66</v>
@@ -46534,7 +46531,7 @@
         <v>3423</v>
       </c>
       <c r="E1165" t="s">
-        <v>3970</v>
+        <v>3966</v>
       </c>
       <c r="F1165" t="s">
         <v>10</v>
@@ -46543,15 +46540,15 @@
         <v>10</v>
       </c>
       <c r="H1165" t="s">
-        <v>3970</v>
+        <v>3966</v>
       </c>
       <c r="I1165" t="s">
-        <v>3971</v>
+        <v>3967</v>
       </c>
     </row>
     <row r="1166" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1166" t="s">
-        <v>3972</v>
+        <v>3968</v>
       </c>
       <c r="B1166" t="s">
         <v>66</v>
@@ -46563,7 +46560,7 @@
         <v>3423</v>
       </c>
       <c r="E1166" t="s">
-        <v>3970</v>
+        <v>3966</v>
       </c>
       <c r="F1166" t="s">
         <v>10</v>
@@ -46572,15 +46569,15 @@
         <v>10</v>
       </c>
       <c r="H1166" t="s">
-        <v>3970</v>
+        <v>3966</v>
       </c>
       <c r="I1166" t="s">
-        <v>3973</v>
+        <v>3969</v>
       </c>
     </row>
     <row r="1167" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1167" t="s">
-        <v>3974</v>
+        <v>3970</v>
       </c>
       <c r="B1167" t="s">
         <v>66</v>
@@ -46589,27 +46586,27 @@
         <v>67</v>
       </c>
       <c r="D1167" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="E1167" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="F1167" t="s">
-        <v>3976</v>
+        <v>3972</v>
       </c>
       <c r="G1167" t="s">
         <v>10</v>
       </c>
       <c r="H1167" t="s">
-        <v>3977</v>
+        <v>3973</v>
       </c>
       <c r="I1167" t="s">
-        <v>3977</v>
+        <v>3973</v>
       </c>
     </row>
     <row r="1168" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1168" t="s">
-        <v>3978</v>
+        <v>3974</v>
       </c>
       <c r="B1168" t="s">
         <v>66</v>
@@ -46618,27 +46615,27 @@
         <v>67</v>
       </c>
       <c r="D1168" t="s">
+        <v>3971</v>
+      </c>
+      <c r="E1168" t="s">
+        <v>3971</v>
+      </c>
+      <c r="F1168" t="s">
         <v>3975</v>
       </c>
-      <c r="E1168" t="s">
-        <v>3975</v>
-      </c>
-      <c r="F1168" t="s">
-        <v>3979</v>
-      </c>
       <c r="G1168" t="s">
         <v>10</v>
       </c>
       <c r="H1168" t="s">
-        <v>3980</v>
+        <v>3976</v>
       </c>
       <c r="I1168" t="s">
-        <v>3980</v>
+        <v>3976</v>
       </c>
     </row>
     <row r="1169" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1169" t="s">
-        <v>3981</v>
+        <v>3977</v>
       </c>
       <c r="B1169" t="s">
         <v>66</v>
@@ -46647,27 +46644,27 @@
         <v>67</v>
       </c>
       <c r="D1169" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="E1169" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="F1169" t="s">
-        <v>3982</v>
+        <v>3978</v>
       </c>
       <c r="G1169" t="s">
         <v>10</v>
       </c>
       <c r="H1169" t="s">
-        <v>3983</v>
+        <v>3979</v>
       </c>
       <c r="I1169" t="s">
-        <v>3983</v>
+        <v>3979</v>
       </c>
     </row>
     <row r="1170" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1170" t="s">
-        <v>3984</v>
+        <v>3980</v>
       </c>
       <c r="B1170" t="s">
         <v>66</v>
@@ -46676,27 +46673,27 @@
         <v>67</v>
       </c>
       <c r="D1170" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="E1170" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="F1170" t="s">
-        <v>3985</v>
+        <v>3981</v>
       </c>
       <c r="G1170" t="s">
         <v>10</v>
       </c>
       <c r="H1170" t="s">
-        <v>3986</v>
+        <v>3982</v>
       </c>
       <c r="I1170" t="s">
-        <v>3986</v>
+        <v>3982</v>
       </c>
     </row>
     <row r="1171" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1171" t="s">
-        <v>3987</v>
+        <v>3983</v>
       </c>
       <c r="B1171" t="s">
         <v>66</v>
@@ -46705,27 +46702,27 @@
         <v>67</v>
       </c>
       <c r="D1171" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="E1171" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="F1171" t="s">
-        <v>3988</v>
+        <v>3984</v>
       </c>
       <c r="G1171" t="s">
         <v>10</v>
       </c>
       <c r="H1171" t="s">
-        <v>3989</v>
+        <v>3985</v>
       </c>
       <c r="I1171" t="s">
-        <v>3989</v>
+        <v>3985</v>
       </c>
     </row>
     <row r="1172" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1172" t="s">
-        <v>3990</v>
+        <v>3986</v>
       </c>
       <c r="B1172" t="s">
         <v>66</v>
@@ -46734,27 +46731,27 @@
         <v>67</v>
       </c>
       <c r="D1172" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="E1172" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="F1172" t="s">
-        <v>3991</v>
+        <v>3987</v>
       </c>
       <c r="G1172" t="s">
         <v>10</v>
       </c>
       <c r="H1172" t="s">
-        <v>3992</v>
+        <v>3988</v>
       </c>
       <c r="I1172" t="s">
-        <v>3992</v>
+        <v>3988</v>
       </c>
     </row>
     <row r="1173" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1173" t="s">
-        <v>3993</v>
+        <v>3989</v>
       </c>
       <c r="B1173" t="s">
         <v>66</v>
@@ -46763,27 +46760,27 @@
         <v>67</v>
       </c>
       <c r="D1173" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="E1173" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="F1173" t="s">
-        <v>3994</v>
+        <v>3990</v>
       </c>
       <c r="G1173" t="s">
         <v>10</v>
       </c>
       <c r="H1173" t="s">
-        <v>3995</v>
+        <v>3991</v>
       </c>
       <c r="I1173" t="s">
-        <v>3995</v>
+        <v>3991</v>
       </c>
     </row>
     <row r="1174" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1174" t="s">
-        <v>3996</v>
+        <v>3992</v>
       </c>
       <c r="B1174" t="s">
         <v>66</v>
@@ -46792,27 +46789,27 @@
         <v>67</v>
       </c>
       <c r="D1174" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="E1174" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="F1174" t="s">
-        <v>3997</v>
+        <v>3993</v>
       </c>
       <c r="G1174" t="s">
         <v>10</v>
       </c>
       <c r="H1174" t="s">
-        <v>3998</v>
+        <v>3994</v>
       </c>
       <c r="I1174" t="s">
-        <v>3998</v>
+        <v>3994</v>
       </c>
     </row>
     <row r="1175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1175" t="s">
-        <v>3999</v>
+        <v>3995</v>
       </c>
       <c r="B1175" t="s">
         <v>66</v>
@@ -46821,27 +46818,27 @@
         <v>67</v>
       </c>
       <c r="D1175" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="E1175" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="F1175" t="s">
-        <v>4000</v>
+        <v>3996</v>
       </c>
       <c r="G1175" t="s">
         <v>10</v>
       </c>
       <c r="H1175" t="s">
-        <v>4001</v>
+        <v>3997</v>
       </c>
       <c r="I1175" t="s">
-        <v>4001</v>
+        <v>3997</v>
       </c>
     </row>
     <row r="1176" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1176" t="s">
-        <v>4002</v>
+        <v>3998</v>
       </c>
       <c r="B1176" t="s">
         <v>66</v>
@@ -46850,27 +46847,27 @@
         <v>67</v>
       </c>
       <c r="D1176" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="E1176" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="F1176" t="s">
-        <v>4003</v>
+        <v>3999</v>
       </c>
       <c r="G1176" t="s">
         <v>10</v>
       </c>
       <c r="H1176" t="s">
-        <v>4004</v>
+        <v>4000</v>
       </c>
       <c r="I1176" t="s">
-        <v>4004</v>
+        <v>4000</v>
       </c>
     </row>
     <row r="1177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1177" t="s">
-        <v>4005</v>
+        <v>4001</v>
       </c>
       <c r="B1177" t="s">
         <v>66</v>
@@ -46879,27 +46876,27 @@
         <v>67</v>
       </c>
       <c r="D1177" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="E1177" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="F1177" t="s">
-        <v>4006</v>
+        <v>4002</v>
       </c>
       <c r="G1177" t="s">
         <v>10</v>
       </c>
       <c r="H1177" t="s">
-        <v>4007</v>
+        <v>4003</v>
       </c>
       <c r="I1177" t="s">
-        <v>4007</v>
+        <v>4003</v>
       </c>
     </row>
     <row r="1178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1178" t="s">
-        <v>4008</v>
+        <v>4004</v>
       </c>
       <c r="B1178" t="s">
         <v>66</v>
@@ -46908,27 +46905,27 @@
         <v>67</v>
       </c>
       <c r="D1178" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="E1178" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="F1178" t="s">
-        <v>4009</v>
+        <v>4005</v>
       </c>
       <c r="G1178" t="s">
         <v>10</v>
       </c>
       <c r="H1178" t="s">
-        <v>4010</v>
+        <v>4006</v>
       </c>
       <c r="I1178" t="s">
-        <v>4010</v>
+        <v>4006</v>
       </c>
     </row>
     <row r="1179" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1179" t="s">
-        <v>4011</v>
+        <v>4007</v>
       </c>
       <c r="B1179" t="s">
         <v>66</v>
@@ -46937,27 +46934,27 @@
         <v>67</v>
       </c>
       <c r="D1179" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="E1179" t="s">
-        <v>3975</v>
+        <v>3971</v>
       </c>
       <c r="F1179" t="s">
-        <v>4012</v>
+        <v>4008</v>
       </c>
       <c r="G1179" t="s">
         <v>10</v>
       </c>
       <c r="H1179" t="s">
-        <v>4013</v>
+        <v>4009</v>
       </c>
       <c r="I1179" t="s">
-        <v>4013</v>
+        <v>4009</v>
       </c>
     </row>
     <row r="1180" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1180" t="s">
-        <v>4014</v>
+        <v>4010</v>
       </c>
       <c r="B1180" t="s">
         <v>66</v>
@@ -46966,27 +46963,27 @@
         <v>67</v>
       </c>
       <c r="D1180" t="s">
+        <v>3971</v>
+      </c>
+      <c r="E1180" t="s">
+        <v>3971</v>
+      </c>
+      <c r="F1180" t="s">
         <v>3975</v>
       </c>
-      <c r="E1180" t="s">
-        <v>3975</v>
-      </c>
-      <c r="F1180" t="s">
-        <v>3979</v>
-      </c>
       <c r="G1180" t="s">
         <v>10</v>
       </c>
       <c r="H1180" t="s">
-        <v>3980</v>
+        <v>3976</v>
       </c>
       <c r="I1180" t="s">
-        <v>4015</v>
+        <v>4011</v>
       </c>
     </row>
     <row r="1181" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1181" t="s">
-        <v>4016</v>
+        <v>4012</v>
       </c>
       <c r="B1181" t="s">
         <v>66</v>
@@ -46998,24 +46995,24 @@
         <v>3423</v>
       </c>
       <c r="E1181" t="s">
-        <v>4017</v>
+        <v>4013</v>
       </c>
       <c r="F1181" t="s">
-        <v>4018</v>
+        <v>4014</v>
       </c>
       <c r="G1181" t="s">
         <v>10</v>
       </c>
       <c r="H1181" t="s">
-        <v>4017</v>
+        <v>4013</v>
       </c>
       <c r="I1181" t="s">
-        <v>4017</v>
+        <v>4013</v>
       </c>
     </row>
     <row r="1182" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1182" t="s">
-        <v>4019</v>
+        <v>4015</v>
       </c>
       <c r="B1182" t="s">
         <v>66</v>
@@ -47027,7 +47024,7 @@
         <v>3423</v>
       </c>
       <c r="E1182" t="s">
-        <v>4020</v>
+        <v>4016</v>
       </c>
       <c r="F1182" t="s">
         <v>10</v>
@@ -47036,15 +47033,15 @@
         <v>10</v>
       </c>
       <c r="H1182" t="s">
-        <v>4020</v>
+        <v>4016</v>
       </c>
       <c r="I1182" t="s">
-        <v>4020</v>
+        <v>4016</v>
       </c>
     </row>
     <row r="1183" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1183" t="s">
-        <v>4021</v>
+        <v>4017</v>
       </c>
       <c r="B1183" t="s">
         <v>66</v>
@@ -47056,24 +47053,24 @@
         <v>3423</v>
       </c>
       <c r="E1183" t="s">
-        <v>4022</v>
+        <v>4018</v>
       </c>
       <c r="F1183" t="s">
-        <v>4023</v>
+        <v>4019</v>
       </c>
       <c r="G1183" t="s">
         <v>10</v>
       </c>
       <c r="H1183" t="s">
-        <v>4024</v>
+        <v>4020</v>
       </c>
       <c r="I1183" t="s">
-        <v>4024</v>
+        <v>4021</v>
       </c>
     </row>
     <row r="1184" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1184" t="s">
-        <v>4025</v>
+        <v>4022</v>
       </c>
       <c r="B1184" t="s">
         <v>66</v>
@@ -47085,7 +47082,7 @@
         <v>3423</v>
       </c>
       <c r="E1184" t="s">
-        <v>4026</v>
+        <v>4023</v>
       </c>
       <c r="F1184" t="s">
         <v>10</v>
@@ -47094,15 +47091,15 @@
         <v>10</v>
       </c>
       <c r="H1184" t="s">
-        <v>4026</v>
+        <v>4023</v>
       </c>
       <c r="I1184" t="s">
-        <v>4027</v>
+        <v>4024</v>
       </c>
     </row>
     <row r="1185" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1185" t="s">
-        <v>4028</v>
+        <v>4025</v>
       </c>
       <c r="B1185" t="s">
         <v>66</v>
@@ -47114,16 +47111,16 @@
         <v>3423</v>
       </c>
       <c r="E1185" t="s">
-        <v>4029</v>
+        <v>4026</v>
       </c>
       <c r="F1185" t="s">
-        <v>4030</v>
+        <v>4027</v>
       </c>
       <c r="G1185" t="s">
         <v>10</v>
       </c>
       <c r="H1185" t="s">
-        <v>4031</v>
+        <v>4028</v>
       </c>
       <c r="I1185" t="s">
         <v>4029</v>
@@ -47131,7 +47128,7 @@
     </row>
     <row r="1186" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1186" t="s">
-        <v>4032</v>
+        <v>4030</v>
       </c>
       <c r="B1186" t="s">
         <v>66</v>
@@ -47143,16 +47140,16 @@
         <v>3423</v>
       </c>
       <c r="E1186" t="s">
-        <v>4033</v>
+        <v>4026</v>
       </c>
       <c r="F1186" t="s">
-        <v>4034</v>
+        <v>4031</v>
       </c>
       <c r="G1186" t="s">
         <v>10</v>
       </c>
       <c r="H1186" t="s">
-        <v>4035</v>
+        <v>4032</v>
       </c>
       <c r="I1186" t="s">
         <v>4033</v>
@@ -47160,7 +47157,7 @@
     </row>
     <row r="1187" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1187" t="s">
-        <v>4036</v>
+        <v>4034</v>
       </c>
       <c r="B1187" t="s">
         <v>66</v>
@@ -47172,7 +47169,7 @@
         <v>3423</v>
       </c>
       <c r="E1187" t="s">
-        <v>4037</v>
+        <v>4035</v>
       </c>
       <c r="F1187" t="s">
         <v>10</v>
@@ -47181,15 +47178,15 @@
         <v>10</v>
       </c>
       <c r="H1187" t="s">
-        <v>4037</v>
+        <v>4035</v>
       </c>
       <c r="I1187" t="s">
-        <v>4037</v>
+        <v>4035</v>
       </c>
     </row>
     <row r="1188" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1188" t="s">
-        <v>4038</v>
+        <v>4036</v>
       </c>
       <c r="B1188" t="s">
         <v>120</v>
@@ -47213,12 +47210,12 @@
         <v>2450</v>
       </c>
       <c r="I1188" t="s">
-        <v>4039</v>
+        <v>4037</v>
       </c>
     </row>
     <row r="1189" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1189" t="s">
-        <v>4040</v>
+        <v>4038</v>
       </c>
       <c r="B1189" t="s">
         <v>120</v>
@@ -47242,12 +47239,12 @@
         <v>2450</v>
       </c>
       <c r="I1189" t="s">
-        <v>4041</v>
+        <v>4039</v>
       </c>
     </row>
     <row r="1190" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1190" t="s">
-        <v>4042</v>
+        <v>4040</v>
       </c>
       <c r="B1190" t="s">
         <v>120</v>
@@ -47271,12 +47268,12 @@
         <v>2450</v>
       </c>
       <c r="I1190" t="s">
-        <v>4043</v>
+        <v>4041</v>
       </c>
     </row>
     <row r="1191" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1191" t="s">
-        <v>4044</v>
+        <v>4042</v>
       </c>
       <c r="B1191" t="s">
         <v>120</v>
@@ -47300,12 +47297,12 @@
         <v>2450</v>
       </c>
       <c r="I1191" t="s">
-        <v>4045</v>
+        <v>4043</v>
       </c>
     </row>
     <row r="1192" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1192" t="s">
-        <v>4046</v>
+        <v>4044</v>
       </c>
       <c r="B1192" t="s">
         <v>66</v>
@@ -47317,7 +47314,7 @@
         <v>3423</v>
       </c>
       <c r="E1192" t="s">
-        <v>4047</v>
+        <v>4045</v>
       </c>
       <c r="F1192" t="s">
         <v>10</v>
@@ -47326,15 +47323,15 @@
         <v>10</v>
       </c>
       <c r="H1192" t="s">
-        <v>4047</v>
+        <v>4045</v>
       </c>
       <c r="I1192" t="s">
-        <v>4047</v>
+        <v>4045</v>
       </c>
     </row>
     <row r="1193" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1193" t="s">
-        <v>4048</v>
+        <v>4046</v>
       </c>
       <c r="B1193" t="s">
         <v>66</v>
@@ -47346,7 +47343,7 @@
         <v>3423</v>
       </c>
       <c r="E1193" t="s">
-        <v>4049</v>
+        <v>4047</v>
       </c>
       <c r="F1193" t="s">
         <v>10</v>
@@ -47355,15 +47352,15 @@
         <v>10</v>
       </c>
       <c r="H1193" t="s">
-        <v>4049</v>
+        <v>4047</v>
       </c>
       <c r="I1193" t="s">
-        <v>4049</v>
+        <v>4047</v>
       </c>
     </row>
     <row r="1194" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1194" t="s">
-        <v>4050</v>
+        <v>4048</v>
       </c>
       <c r="B1194" t="s">
         <v>66</v>
@@ -47375,7 +47372,7 @@
         <v>3423</v>
       </c>
       <c r="E1194" t="s">
-        <v>4051</v>
+        <v>4049</v>
       </c>
       <c r="F1194" t="s">
         <v>10</v>
@@ -47384,15 +47381,15 @@
         <v>10</v>
       </c>
       <c r="H1194" t="s">
-        <v>4051</v>
+        <v>4049</v>
       </c>
       <c r="I1194" t="s">
-        <v>4051</v>
+        <v>4049</v>
       </c>
     </row>
     <row r="1195" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1195" t="s">
-        <v>4052</v>
+        <v>4050</v>
       </c>
       <c r="B1195" t="s">
         <v>66</v>
@@ -47404,7 +47401,7 @@
         <v>3423</v>
       </c>
       <c r="E1195" t="s">
-        <v>4053</v>
+        <v>4051</v>
       </c>
       <c r="F1195" t="s">
         <v>10</v>
@@ -47413,15 +47410,15 @@
         <v>10</v>
       </c>
       <c r="H1195" t="s">
-        <v>4053</v>
+        <v>4051</v>
       </c>
       <c r="I1195" t="s">
-        <v>4053</v>
+        <v>4051</v>
       </c>
     </row>
     <row r="1196" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1196" t="s">
-        <v>4054</v>
+        <v>4052</v>
       </c>
       <c r="B1196" t="s">
         <v>66</v>
@@ -47433,24 +47430,24 @@
         <v>3423</v>
       </c>
       <c r="E1196" t="s">
+        <v>4053</v>
+      </c>
+      <c r="F1196" t="s">
+        <v>2949</v>
+      </c>
+      <c r="G1196" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1196" t="s">
+        <v>4054</v>
+      </c>
+      <c r="I1196" t="s">
         <v>4055</v>
-      </c>
-      <c r="F1196" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1196" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1196" t="s">
-        <v>4055</v>
-      </c>
-      <c r="I1196" t="s">
-        <v>4056</v>
       </c>
     </row>
     <row r="1197" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1197" t="s">
-        <v>4057</v>
+        <v>4056</v>
       </c>
       <c r="B1197" t="s">
         <v>66</v>
@@ -47462,24 +47459,24 @@
         <v>3423</v>
       </c>
       <c r="E1197" t="s">
-        <v>4058</v>
+        <v>4053</v>
       </c>
       <c r="F1197" t="s">
-        <v>10</v>
+        <v>1055</v>
       </c>
       <c r="G1197" t="s">
         <v>10</v>
       </c>
       <c r="H1197" t="s">
-        <v>4058</v>
+        <v>4057</v>
       </c>
       <c r="I1197" t="s">
-        <v>4058</v>
+        <v>4057</v>
       </c>
     </row>
     <row r="1198" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1198" t="s">
-        <v>4059</v>
+        <v>4058</v>
       </c>
       <c r="B1198" t="s">
         <v>66</v>
@@ -47491,24 +47488,24 @@
         <v>3423</v>
       </c>
       <c r="E1198" t="s">
+        <v>4059</v>
+      </c>
+      <c r="F1198" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1198" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1198" t="s">
+        <v>4059</v>
+      </c>
+      <c r="I1198" t="s">
         <v>4060</v>
-      </c>
-      <c r="F1198" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1198" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1198" t="s">
-        <v>4060</v>
-      </c>
-      <c r="I1198" t="s">
-        <v>4061</v>
       </c>
     </row>
     <row r="1199" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1199" t="s">
-        <v>4062</v>
+        <v>4061</v>
       </c>
       <c r="B1199" t="s">
         <v>66</v>
@@ -47520,24 +47517,24 @@
         <v>3423</v>
       </c>
       <c r="E1199" t="s">
-        <v>4063</v>
+        <v>4062</v>
       </c>
       <c r="F1199" t="s">
-        <v>3730</v>
+        <v>3729</v>
       </c>
       <c r="G1199" t="s">
         <v>10</v>
       </c>
       <c r="H1199" t="s">
-        <v>4063</v>
+        <v>4062</v>
       </c>
       <c r="I1199" t="s">
-        <v>4063</v>
+        <v>4062</v>
       </c>
     </row>
     <row r="1200" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1200" t="s">
-        <v>4064</v>
+        <v>4063</v>
       </c>
       <c r="B1200" t="s">
         <v>66</v>
@@ -47549,24 +47546,24 @@
         <v>3423</v>
       </c>
       <c r="E1200" t="s">
+        <v>4064</v>
+      </c>
+      <c r="F1200" t="s">
+        <v>10</v>
+      </c>
+      <c r="G1200" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1200" t="s">
+        <v>4064</v>
+      </c>
+      <c r="I1200" t="s">
         <v>4065</v>
-      </c>
-      <c r="F1200" t="s">
-        <v>10</v>
-      </c>
-      <c r="G1200" t="s">
-        <v>10</v>
-      </c>
-      <c r="H1200" t="s">
-        <v>4065</v>
-      </c>
-      <c r="I1200" t="s">
-        <v>4066</v>
       </c>
     </row>
     <row r="1201" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1201" t="s">
-        <v>4067</v>
+        <v>4066</v>
       </c>
       <c r="B1201" t="s">
         <v>2841</v>
@@ -47587,15 +47584,15 @@
         <v>3104</v>
       </c>
       <c r="H1201" t="s">
-        <v>4068</v>
+        <v>4067</v>
       </c>
       <c r="I1201" t="s">
-        <v>4068</v>
+        <v>4067</v>
       </c>
     </row>
     <row r="1202" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1202" t="s">
-        <v>4069</v>
+        <v>4068</v>
       </c>
       <c r="B1202" t="s">
         <v>2841</v>
@@ -47616,15 +47613,15 @@
         <v>3097</v>
       </c>
       <c r="H1202" t="s">
-        <v>4070</v>
+        <v>4069</v>
       </c>
       <c r="I1202" t="s">
-        <v>4070</v>
+        <v>4069</v>
       </c>
     </row>
     <row r="1203" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1203" t="s">
-        <v>4071</v>
+        <v>4070</v>
       </c>
       <c r="B1203" t="s">
         <v>120</v>
@@ -47642,18 +47639,18 @@
         <v>2216</v>
       </c>
       <c r="G1203" t="s">
+        <v>4071</v>
+      </c>
+      <c r="H1203" t="s">
         <v>4072</v>
       </c>
-      <c r="H1203" t="s">
-        <v>4073</v>
-      </c>
       <c r="I1203" t="s">
-        <v>4073</v>
+        <v>4072</v>
       </c>
     </row>
     <row r="1204" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1204" t="s">
-        <v>4074</v>
+        <v>4073</v>
       </c>
       <c r="B1204" t="s">
         <v>2841</v>
@@ -47674,15 +47671,15 @@
         <v>3097</v>
       </c>
       <c r="H1204" t="s">
-        <v>4075</v>
+        <v>4074</v>
       </c>
       <c r="I1204" t="s">
-        <v>4075</v>
+        <v>4074</v>
       </c>
     </row>
     <row r="1205" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1205" t="s">
-        <v>4076</v>
+        <v>4075</v>
       </c>
       <c r="B1205" t="s">
         <v>2841</v>
@@ -47703,10 +47700,10 @@
         <v>3097</v>
       </c>
       <c r="H1205" t="s">
-        <v>4077</v>
+        <v>4076</v>
       </c>
       <c r="I1205" t="s">
-        <v>4077</v>
+        <v>4076</v>
       </c>
     </row>
   </sheetData>
@@ -47727,18 +47724,18 @@
   <sheetData>
     <row r="1" spans="1:3" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>4078</v>
+        <v>4077</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>4079</v>
+        <v>4078</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4080</v>
+        <v>4079</v>
       </c>
       <c r="B2" t="s">
         <v>24</v>
@@ -47749,18 +47746,18 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4081</v>
+        <v>4080</v>
       </c>
       <c r="B3" t="s">
         <v>176</v>
       </c>
       <c r="C3" t="s">
-        <v>4082</v>
+        <v>4081</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4083</v>
+        <v>4082</v>
       </c>
       <c r="B4" t="s">
         <v>14</v>
@@ -47771,7 +47768,7 @@
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>4084</v>
+        <v>4083</v>
       </c>
       <c r="B5" t="s">
         <v>14</v>
@@ -47782,7 +47779,7 @@
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>4085</v>
+        <v>4084</v>
       </c>
       <c r="B6" t="s">
         <v>1097</v>
@@ -47793,7 +47790,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>4086</v>
+        <v>4085</v>
       </c>
       <c r="B7" t="s">
         <v>120</v>
@@ -47804,7 +47801,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>4087</v>
+        <v>4086</v>
       </c>
       <c r="B8" t="s">
         <v>120</v>
@@ -47815,7 +47812,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>4088</v>
+        <v>4087</v>
       </c>
       <c r="B9" t="s">
         <v>2841</v>
@@ -47826,7 +47823,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>4089</v>
+        <v>4088</v>
       </c>
       <c r="B10" t="s">
         <v>899</v>
@@ -47837,7 +47834,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>4090</v>
+        <v>4089</v>
       </c>
       <c r="B11" t="s">
         <v>66</v>
@@ -47859,34 +47856,34 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>4090</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>4091</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>4092</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>4092</v>
+      </c>
+      <c r="B2" t="s">
         <v>4093</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4094</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>4094</v>
+      </c>
+      <c r="B3" t="s">
         <v>4095</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4096</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>4096</v>
+      </c>
+      <c r="B4" t="s">
         <v>4097</v>
-      </c>
-      <c r="B4" t="s">
-        <v>4098</v>
       </c>
     </row>
   </sheetData>
@@ -47908,7 +47905,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>4099</v>
+        <v>4098</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
@@ -47919,7 +47916,7 @@
         <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>4100</v>
+        <v>4099</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
@@ -47930,7 +47927,7 @@
         <v>24</v>
       </c>
       <c r="C3" t="s">
-        <v>4101</v>
+        <v>4100</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
@@ -47941,7 +47938,7 @@
         <v>176</v>
       </c>
       <c r="C4" t="s">
-        <v>4102</v>
+        <v>4101</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
@@ -47952,7 +47949,7 @@
         <v>14</v>
       </c>
       <c r="C5" t="s">
-        <v>4103</v>
+        <v>4102</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -47963,7 +47960,7 @@
         <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>4104</v>
+        <v>4103</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -47974,7 +47971,7 @@
         <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>4105</v>
+        <v>4104</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -47985,7 +47982,7 @@
         <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>4106</v>
+        <v>4105</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -47996,7 +47993,7 @@
         <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>4107</v>
+        <v>4106</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
@@ -48007,7 +48004,7 @@
         <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>4108</v>
+        <v>4107</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
@@ -48018,7 +48015,7 @@
         <v>899</v>
       </c>
       <c r="C11" t="s">
-        <v>4109</v>
+        <v>4108</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
@@ -48029,7 +48026,7 @@
         <v>899</v>
       </c>
       <c r="C12" t="s">
-        <v>4110</v>
+        <v>4109</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
@@ -48040,7 +48037,7 @@
         <v>899</v>
       </c>
       <c r="C13" t="s">
-        <v>4111</v>
+        <v>4110</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
@@ -48051,7 +48048,7 @@
         <v>1097</v>
       </c>
       <c r="C14" t="s">
-        <v>4112</v>
+        <v>4111</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -48062,7 +48059,7 @@
         <v>2841</v>
       </c>
       <c r="C15" t="s">
-        <v>4113</v>
+        <v>4112</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -48073,7 +48070,7 @@
         <v>120</v>
       </c>
       <c r="C16" t="s">
-        <v>4114</v>
+        <v>4113</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -48084,7 +48081,7 @@
         <v>120</v>
       </c>
       <c r="C17" t="s">
-        <v>4115</v>
+        <v>4114</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
@@ -48095,7 +48092,7 @@
         <v>120</v>
       </c>
       <c r="C18" t="s">
-        <v>4116</v>
+        <v>4115</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -48106,7 +48103,7 @@
         <v>66</v>
       </c>
       <c r="C19" t="s">
-        <v>4117</v>
+        <v>4116</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
@@ -48117,7 +48114,7 @@
         <v>66</v>
       </c>
       <c r="C20" t="s">
-        <v>4118</v>
+        <v>4117</v>
       </c>
     </row>
   </sheetData>

</xml_diff>